<commit_message>
Deploy PDF format exports for Form A and Form B with embedded logos and borders
</commit_message>
<xml_diff>
--- a/Ready_To_Print_OSDS-NSTP-Form-2-A.xlsx
+++ b/Ready_To_Print_OSDS-NSTP-Form-2-A.xlsx
@@ -567,7 +567,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:Z18"/>
+  <dimension ref="A1:Z19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1019,18 +1019,102 @@
         <v>25</v>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="13" t="inlineStr">
+    <row r="16" ht="20" customHeight="1">
+      <c r="A16" s="11" t="inlineStr">
+        <is>
+          <t>CVSU BACOOR</t>
+        </is>
+      </c>
+      <c r="B16" s="11" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="C16" s="12" t="n">
+        <v>30</v>
+      </c>
+      <c r="D16" s="12" t="n">
+        <v>10</v>
+      </c>
+      <c r="E16" s="12" t="n">
+        <v>90</v>
+      </c>
+      <c r="F16" s="12" t="n">
+        <v>110</v>
+      </c>
+      <c r="G16" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="I16" s="12" t="n">
+        <v>30</v>
+      </c>
+      <c r="J16" s="12" t="n">
+        <v>10</v>
+      </c>
+      <c r="K16" s="12" t="n">
+        <v>88</v>
+      </c>
+      <c r="L16" s="12" t="n">
+        <v>108</v>
+      </c>
+      <c r="M16" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="N16" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="O16" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="P16" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q16" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="R16" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="S16" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="T16" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="U16" s="12" t="n">
+        <v>30</v>
+      </c>
+      <c r="V16" s="12" t="n">
+        <v>10</v>
+      </c>
+      <c r="W16" s="12" t="n">
+        <v>88</v>
+      </c>
+      <c r="X16" s="12" t="n">
+        <v>108</v>
+      </c>
+      <c r="Y16" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z16" s="12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="13" t="inlineStr">
         <is>
           <t>Prepared by: NSTP Department Coordinator</t>
         </is>
       </c>
-      <c r="J18" s="13" t="inlineStr">
+      <c r="J19" s="13" t="inlineStr">
         <is>
           <t>Verified by: Campus NSTP Director</t>
         </is>
       </c>
-      <c r="T18" s="13" t="inlineStr">
+      <c r="T19" s="13" t="inlineStr">
         <is>
           <t>Approved by: Campus Administrator</t>
         </is>

</xml_diff>

<commit_message>
Comprehensive audit, cleanup, security verification, and 5-section documentation update
</commit_message>
<xml_diff>
--- a/Ready_To_Print_OSDS-NSTP-Form-2-A.xlsx
+++ b/Ready_To_Print_OSDS-NSTP-Form-2-A.xlsx
@@ -567,7 +567,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:Z19"/>
+  <dimension ref="A1:Z18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1019,102 +1019,18 @@
         <v>25</v>
       </c>
     </row>
-    <row r="16" ht="20" customHeight="1">
-      <c r="A16" s="11" t="inlineStr">
-        <is>
-          <t>CVSU BACOOR</t>
-        </is>
-      </c>
-      <c r="B16" s="11" t="inlineStr">
-        <is>
-          <t>PUBLIC</t>
-        </is>
-      </c>
-      <c r="C16" s="12" t="n">
-        <v>30</v>
-      </c>
-      <c r="D16" s="12" t="n">
-        <v>10</v>
-      </c>
-      <c r="E16" s="12" t="n">
-        <v>90</v>
-      </c>
-      <c r="F16" s="12" t="n">
-        <v>110</v>
-      </c>
-      <c r="G16" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="H16" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="I16" s="12" t="n">
-        <v>30</v>
-      </c>
-      <c r="J16" s="12" t="n">
-        <v>10</v>
-      </c>
-      <c r="K16" s="12" t="n">
-        <v>88</v>
-      </c>
-      <c r="L16" s="12" t="n">
-        <v>108</v>
-      </c>
-      <c r="M16" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="N16" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="O16" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="P16" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q16" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="R16" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="S16" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="T16" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="U16" s="12" t="n">
-        <v>30</v>
-      </c>
-      <c r="V16" s="12" t="n">
-        <v>10</v>
-      </c>
-      <c r="W16" s="12" t="n">
-        <v>88</v>
-      </c>
-      <c r="X16" s="12" t="n">
-        <v>108</v>
-      </c>
-      <c r="Y16" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z16" s="12" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="13" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="13" t="inlineStr">
         <is>
           <t>Prepared by: NSTP Department Coordinator</t>
         </is>
       </c>
-      <c r="J19" s="13" t="inlineStr">
+      <c r="J18" s="13" t="inlineStr">
         <is>
           <t>Verified by: Campus NSTP Director</t>
         </is>
       </c>
-      <c r="T19" s="13" t="inlineStr">
+      <c r="T18" s="13" t="inlineStr">
         <is>
           <t>Approved by: Campus Administrator</t>
         </is>

</xml_diff>